<commit_message>
Lightning matching: condition picker with range calendar, candidate list, selection and application flow
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QdvtKC2X7yNk6ULcR3oaXd
</commit_message>
<xml_diff>
--- a/templates/관리사_데이터_양식.xlsx
+++ b/templates/관리사_데이터_양식.xlsx
@@ -195,6 +195,71 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>따사로운</author>
+  </authors>
+  <commentList>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>연령대(50대/60대) 판단에만 사용, 외부에 공개되지 않음 (예: 1975-03-02)</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>시·구 단위, 쉼표로 구분. 예) 서울 강남구, 서울 서초구</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>예) 월화수목금 (현재 매칭 조건에는 미사용, 상담 시 참고)</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>예) 2026-11-01~2026-11-20, 2026-12-24~2026-12-26 (쉼표로 여러 개)</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>지금 배정 중이면 종료일. 이 날짜 이후부터 매칭 가능</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>쉼표로 복수 입력 가능: 차분,조용,쾌활·유쾌,사교,전문</t>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="0" shapeId="0">
+      <text>
+        <t>필수. 비어 있거나 일정 종료일 전에 만료되면 매칭 제외 (예: 2027-06-30)</t>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="0" shapeId="0">
+      <text>
+        <t>필수. 비어 있거나 일정 종료일 전에 만료되면 매칭 제외</t>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="0" shapeId="0">
+      <text>
+        <t>필수. 비어 있거나 일정 종료일 전에 만료되면 매칭 제외</t>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="0" shapeId="0">
+      <text>
+        <t>선택. 값이 있고 만료됐을 때만 제외</t>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="0" shapeId="0">
+      <text>
+        <t>수료증·위탁계약·업무협약·개인정보동의 등 완비 여부 Y/N</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -585,7 +650,7 @@
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>활동지역(시·구, 쉼표로 구분)</t>
+          <t>활동지역</t>
         </is>
       </c>
       <c r="M1" s="3" t="inlineStr">
@@ -620,12 +685,12 @@
       </c>
       <c r="S1" s="4" t="inlineStr">
         <is>
-          <t>가능요일(예: 월화수목금)</t>
+          <t>가능요일</t>
         </is>
       </c>
       <c r="T1" s="4" t="inlineStr">
         <is>
-          <t>근무불가기간(예: 11/1~11/20)</t>
+          <t>근무불가기간</t>
         </is>
       </c>
       <c r="U1" s="4" t="inlineStr">
@@ -695,7 +760,7 @@
       </c>
       <c r="AH1" s="7" t="inlineStr">
         <is>
-          <t>서류완비(수료증·위탁계약·협약·개인정보동의 등)</t>
+          <t>서류완비</t>
         </is>
       </c>
       <c r="AI1" s="8" t="inlineStr">
@@ -805,8 +870,6 @@
           <t>월화수목금</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
           <t>쾌활·유쾌</t>
@@ -827,24 +890,14 @@
           <t>5</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="14">
+  <dataValidations count="13">
     <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"활동중,휴식,중단"</formula1>
     </dataValidation>
@@ -881,14 +934,12 @@
     <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"무관,불가,강아지만,고양이만"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"조용,차분,쾌활·유쾌,사교"</formula1>
-    </dataValidation>
     <dataValidation sqref="AH2:AH500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -898,7 +949,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -911,9 +962,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -967,6 +1016,44 @@
       <c r="A10" t="inlineStr">
         <is>
           <t>8. 진단서·범죄경력 원본 서류는 시트에 올리지 말고 만료일/완비 여부만 기록하세요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>■ 번개매칭 연동 규칙 (시트 이름은 반드시 "관리사")</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>· 열 제목(1행)은 바꾸지 마세요. 사이트가 열 제목으로 데이터를 읽습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>· 필수 서류 3종(건강진단서·범죄경력조회·아동학대범죄경력) 만료일이 비었거나 일정 종료일 전에 만료되면 후보에서 제외됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>· 성향은 후보를 거르지 않고 "성향 일치" 표시와 정렬 우선순위에만 반영됩니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>· 고객 화면에는 이름 첫 글자만 보이고, 전화·주소·생년월일은 공개되지 않습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>